<commit_message>
versión para entrega, challegne EDSA
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\edison\Documents\UiPath\ChallengeEDSA_202504\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E881E603-0E71-4DFA-A9A8-05B055EA0175}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23482496-84DF-4F40-AC41-11460EE68FD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6495" yWindow="5640" windowWidth="21600" windowHeight="11385" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="63">
   <si>
     <t>Name</t>
   </si>
@@ -155,15 +155,6 @@
     <t xml:space="preserve">The maximum number of consecutive system exceptions was reached. </t>
   </si>
   <si>
-    <t>LoadQueue</t>
-  </si>
-  <si>
-    <t>TRUE</t>
-  </si>
-  <si>
-    <t>Determina si el proceso debe o no volver a cargar el input con el listado de productos a buscar. True  = Si, False = No</t>
-  </si>
-  <si>
     <t>queue_edsa</t>
   </si>
   <si>
@@ -183,6 +174,45 @@
   </si>
   <si>
     <t>edsa_challenge_precio_menor_a</t>
+  </si>
+  <si>
+    <t>OrchestratorQueueName</t>
+  </si>
+  <si>
+    <t>edsa_challenge_ruta_input_productos</t>
+  </si>
+  <si>
+    <t>ruta_input_productos</t>
+  </si>
+  <si>
+    <t>edsa_challenge_url_amazon</t>
+  </si>
+  <si>
+    <t>url_amazon</t>
+  </si>
+  <si>
+    <t>nombre_proceso</t>
+  </si>
+  <si>
+    <t>edsa_challenge_nombre_proceso</t>
+  </si>
+  <si>
+    <t>correo_excepcion</t>
+  </si>
+  <si>
+    <t>edsa_challenge_correo_excepcion</t>
+  </si>
+  <si>
+    <t>edsa_challenge_asunto_correo</t>
+  </si>
+  <si>
+    <t>asunto_correo</t>
+  </si>
+  <si>
+    <t>edsa_challenge_calificacion_para_filtrar</t>
+  </si>
+  <si>
+    <t>calificacion_para_filtrar</t>
   </si>
 </sst>
 </file>
@@ -609,10 +639,10 @@
     </row>
     <row r="2" spans="1:26" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>22</v>
@@ -1641,7 +1671,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:Z20"/>
+  <dimension ref="A1:Z19"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="41" customWidth="1"/>
@@ -1836,22 +1866,11 @@
         <v>41</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="30">
-      <c r="A18" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="B18" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="C18" s="6" t="s">
-        <v>45</v>
-      </c>
+    <row r="18" spans="1:3">
+      <c r="C18" s="3"/>
     </row>
     <row r="19" spans="1:3">
       <c r="C19" s="3"/>
-    </row>
-    <row r="20" spans="1:3">
-      <c r="C20" s="3"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2"/>
@@ -1865,7 +1884,7 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="31.85546875" customWidth="1"/>
-    <col min="2" max="2" width="30.140625" customWidth="1"/>
+    <col min="2" max="2" width="36.140625" customWidth="1"/>
     <col min="3" max="3" width="60.28515625" customWidth="1"/>
     <col min="4" max="26" width="65.42578125" customWidth="1"/>
   </cols>
@@ -1908,34 +1927,76 @@
     </row>
     <row r="2" spans="1:26" ht="14.25" customHeight="1">
       <c r="A2" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="B2" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
     </row>
     <row r="3" spans="1:26" ht="14.25" customHeight="1">
       <c r="A3" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="B3" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="4" spans="1:26" ht="14.25" customHeight="1">
       <c r="A4" t="s">
+        <v>48</v>
+      </c>
+      <c r="B4" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="5" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B5" t="s">
         <v>51</v>
       </c>
-      <c r="B4" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="5" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="6" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="7" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="8" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="9" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="10" spans="1:26" ht="14.25" customHeight="1"/>
+    </row>
+    <row r="6" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B6" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="7" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A7" t="s">
+        <v>55</v>
+      </c>
+      <c r="B7" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="8" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A8" t="s">
+        <v>57</v>
+      </c>
+      <c r="B8" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="9" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A9" t="s">
+        <v>60</v>
+      </c>
+      <c r="B9" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="10" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A10" t="s">
+        <v>62</v>
+      </c>
+      <c r="B10" t="s">
+        <v>61</v>
+      </c>
+    </row>
     <row r="11" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="12" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="13" spans="1:26" ht="14.25" customHeight="1"/>

</xml_diff>